<commit_message>
Fix illegal HTML warnings: escape literal XML tags in FSH descriptions with backticks 0a2fcec90de9be5ac7ac9d39e5a4beae9fb5dc58
</commit_message>
<xml_diff>
--- a/fix/qa-validation-errors/ig/StructureDefinition-cisis-telecom.xlsx
+++ b/fix/qa-validation-errors/ig/StructureDefinition-cisis-telecom.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-03T14:38:58+00:00</t>
+    <t>2026-09-04T10:07:56+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,11 +84,11 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Coordonnées télécom : 
+    <t>Coordonnées télécom :
  - Exemples :
-&lt;telecom value='tel:0147150000' use='H'/&gt;
-&lt;telecom value='mailto:adam.homme@fournisseur.fr'/&gt;
-&lt;telecom value='ftp://serveur/dossierdesante/exemple/'/&gt;</t>
+`&lt;telecom value='tel:0147150000' use='H'/&gt;`
+`&lt;telecom value='mailto:adam.homme@fournisseur.fr'/&gt;`
+`&lt;telecom value='ftp://serveur/dossierdesante/exemple/'/&gt;`</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>